<commit_message>
update nmd perturbation dataset info
</commit_message>
<xml_diff>
--- a/data/NMD_Perturbation_TopStudySamples_20260712.xlsx
+++ b/data/NMD_Perturbation_TopStudySamples_20260712.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\aobermayer4\Projects\active\Public_NMD_Perturbation_Data\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://moffitt-my.sharepoint.com/personal/alyssa_obermayer_moffitt_org/Documents/Documents/Projects/Active/NMD_Perturbation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1180FC-E05E-412E-A9C8-872707654177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="13_ncr:1_{5A1180FC-E05E-412E-A9C8-872707654177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBB80609-CB8B-4057-A715-107CBCEA5C66}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
   </bookViews>
   <sheets>
     <sheet name="NMD_Perturbation_TopStudySample" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2232" uniqueCount="770">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2357" uniqueCount="866">
   <si>
     <t>GSE_ID</t>
   </si>
@@ -2205,9 +2205,6 @@
     <t>n control</t>
   </si>
   <si>
-    <t>perturbation</t>
-  </si>
-  <si>
     <t>Seq Type</t>
   </si>
   <si>
@@ -2332,6 +2329,297 @@
   </si>
   <si>
     <t>https://www.ebi.ac.uk/biostudies/ArrayExpress/studies/E-MTAB-13837?query=E-MTAB-13837</t>
+  </si>
+  <si>
+    <t>n ambiguous</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>PRJNA971187</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE232185</t>
+  </si>
+  <si>
+    <t>SRP436870</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE232333</t>
+  </si>
+  <si>
+    <t>PRJNA971629</t>
+  </si>
+  <si>
+    <t>NMD inhibition (NMDi) was achieved by supplementing the medium with 0.3 μM of a SMG1 inhibitor (hSMG1-inhibitor 11e, PC-35788 ProbeChem®)</t>
+  </si>
+  <si>
+    <t>Organism</t>
+  </si>
+  <si>
+    <t>Cell Line</t>
+  </si>
+  <si>
+    <t>HT1080, SMG7KO_11 and SMG7KO_12 cell lines</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>MMP9 overexpression induced</t>
+  </si>
+  <si>
+    <t>HT1080, SMG7KO_12+SMG7(rescue), SMG7KO</t>
+  </si>
+  <si>
+    <t>Perturbation</t>
+  </si>
+  <si>
+    <t>Perturbation Text</t>
+  </si>
+  <si>
+    <t>SRP437288</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE12928</t>
+  </si>
+  <si>
+    <t>PRJNA110847</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10480688/</t>
+  </si>
+  <si>
+    <t>Cell Line Info</t>
+  </si>
+  <si>
+    <t>human fibrosarcoma cell line</t>
+  </si>
+  <si>
+    <t>gastric cancer cell lines</t>
+  </si>
+  <si>
+    <t>GP202, GP220</t>
+  </si>
+  <si>
+    <t>100 nM of siRNA duplexes directed against UPF1 (Dharmacon, Chicago, IL) or non-specific siRNA duplexes (CVII) (Dharmacon) using the lipofectamine 2000 reagent (Invitrogen) according to the manufacturer's instructions</t>
+  </si>
+  <si>
+    <t>The 2 'ambiguous' samples are from: DNA isolated from blood obtained from eighteen healthy males was pooled and used as normal reference</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE30499</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC2709900</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC3165546/</t>
+  </si>
+  <si>
+    <t>PRJNA143335</t>
+  </si>
+  <si>
+    <t>U2OS</t>
+  </si>
+  <si>
+    <t>osteosarcoma cell line</t>
+  </si>
+  <si>
+    <t>Mouse (Xenograft)</t>
+  </si>
+  <si>
+    <t>Total RNA was collected from U2OS cells grown under normoxic conditions, treated with 100 μg/ml emetine or 2.5 μg/ml tunicamycin, or rendered hypoxic for 3 h prior to the addition of DRB and collection of RNA at time zero and at 1.5, 3.0, and 4.5 h</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE305669</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12640816/</t>
+  </si>
+  <si>
+    <t>PRJNA1307433</t>
+  </si>
+  <si>
+    <t>SRP610054</t>
+  </si>
+  <si>
+    <t>HK1, 5-8F and 6-10B</t>
+  </si>
+  <si>
+    <t>nasopharyngeal carcinoma, 5-8F (high metastatic) and 6-10B (low metastatic) are subclones derived from the NPC cell line SUNE1</t>
+  </si>
+  <si>
+    <t>8 samples, 4 in each group, experienced cellular stress conditions, hypoxia, Tunicamycin (inhibit glycoprotein synthesis), For comparisons of NMD targets in normal and neoplastic tissues, expression levels of NMD targets were collected from a compendium of samples of both normal and tumor human tissues (breast, liver, lung, and esophagus) (Gene Expression Omnibus [GEO] accession number GSE5364 [http://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE5364]). Each gene profile was mean centered across the compendium.</t>
+  </si>
+  <si>
+    <t>UPF1 knockdown (UPF1-KD), UPF1-overexpressing, and Emetine-treated NPC cells and their corresponding control cell lines, Considering that the 5-8F and 6-10B cells derived from the same parental line, biological replicates were not used for sequencing of UPF1-KD 6-10B cells, Emetine treated 5-8F cells and their corresponding controls.</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE16856</t>
+  </si>
+  <si>
+    <t>PRJNA117559</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC2749059/</t>
+  </si>
+  <si>
+    <t>LNCaP and 22Rv1</t>
+  </si>
+  <si>
+    <t>prostate carcinoma cell lines</t>
+  </si>
+  <si>
+    <t>Caffeine (10 mM) was added to three plates and one plate was incubated without caffeine as a control, The caffeine-containing medium of the two remaining plates was removed, the cells were washed twice with phosphate-buffered saline and the medium with actinomycin D (2 μg/ml) together with caffeine (10 mM) was added to one plate. Actinomycin D alone was added to the other plate</t>
+  </si>
+  <si>
+    <t>Caffeine</t>
+  </si>
+  <si>
+    <t>GINI method, actinomycin D used to block transcription, During this step, the natural substrate of NMD, including nonsense mutation-containing transcripts, are degraded at different rates between the two plates, depending on the NMD status in each plate, while the stress response genes should be degraded with the same efficiency regardless of NMD status</t>
+  </si>
+  <si>
+    <t>2 inhib, 4 over</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12809107/</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE289050</t>
+  </si>
+  <si>
+    <t>Renal Cell Carcinoma</t>
+  </si>
+  <si>
+    <t>PRJNA1220709</t>
+  </si>
+  <si>
+    <t>SRP562264</t>
+  </si>
+  <si>
+    <t>A-498 (ATCC, HTB-44) and A-704 (ATCC, HTB-45)</t>
+  </si>
+  <si>
+    <t>Differential expression tables for UPF1, UPF2 and MAGOH knock-down vs. wild type were downloaded from ENCODE (https://www.encodeproject.org). Genes with log fold change &gt;2 in each knockdown condition were measured. Genes that changed in at least two knock-down conditions were selected for the NMD signature list.</t>
+  </si>
+  <si>
+    <t>Pladienolide B (100 nM), Sapanisertib (100 nM), Torin2 (300 nM), or hSMG-1 inhibitor 11j (300 nM)</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE24205</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC3162583/</t>
+  </si>
+  <si>
+    <t>PRJNA130181</t>
+  </si>
+  <si>
+    <t>Five families were chosen with 6 affected and 6 healthy controls. Lymphoblastoid cell lines were derived from whole blood</t>
+  </si>
+  <si>
+    <t>Lymphoblastoid cell lines</t>
+  </si>
+  <si>
+    <t>Emetine and UPF1 siRNA, Lentiviral transduction to overexpress UPF1</t>
+  </si>
+  <si>
+    <t>Upf1/Rent1 shRNA, Emetine</t>
+  </si>
+  <si>
+    <t>The emetine treatment protocol was described previously [12]. Briefly, for each cell line, we treated half of the subconfluent cells with 100 μg/ml of emetine dihydrochloride hydrate (Fluka, Buchs, Switzerland) and the rest were used as untreated controls. Both the treated and untreated cells were incubated for 10 h at 37°C. After this, actinomycin D (Sigma-Aldrich) was added to the treated and untreated cells</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE37210</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC3409022/</t>
+  </si>
+  <si>
+    <t>PRJNA158973</t>
+  </si>
+  <si>
+    <t>LCL from 12 individuals</t>
+  </si>
+  <si>
+    <t>LCL from 3 breast cancer families, HT29 (positive control), 2 BRCA positive control LCL</t>
+  </si>
+  <si>
+    <t>Lymphoblastoid cell lines, colon cancer cell line</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE5486</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/1210098</t>
+  </si>
+  <si>
+    <t>MSI+ colon cancer cell lines</t>
+  </si>
+  <si>
+    <t>LS180 (MSI+) and SW480 (MSI-)</t>
+  </si>
+  <si>
+    <t>PRJNA96123</t>
+  </si>
+  <si>
+    <t>Caffeine and Emetine</t>
+  </si>
+  <si>
+    <t>inhibition of NMD with emetine is complemented with inhibiting NMD by blocking the phosphorylation of the hUpf1 protein with caffeine. In addition, to enhance the GINI strategy, comparing mRNA level alterations produced by inhibiting transcription alone or inhbiiting transcription together with NMD following caffeine pretreatment were used for the efficient identification of false positives produced as a result of stress response to NMD inhibition</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC6356069/</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE109143</t>
+  </si>
+  <si>
+    <t>PRJNA429768</t>
+  </si>
+  <si>
+    <t>HEK-293</t>
+  </si>
+  <si>
+    <t>siRNAs against hnRNP L, UPF1, or a non-targeting control (NS).</t>
+  </si>
+  <si>
+    <t>human embryonic kidney cell line</t>
+  </si>
+  <si>
+    <t>In the Tet-Off system, a tetracycline-controlled transactivator (tTA) binds to a responsive promoter and turns target gene transcription ON. When tetracycline (Tc) or its derivative doxycycline (Dox) is added to the culture, it binds to tTA, causing it to detach from the promoter and effectively turning gene expression OFF</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE152436</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC7397857/</t>
+  </si>
+  <si>
+    <t>HeLa</t>
+  </si>
+  <si>
+    <t>UPF1 siRNA, UPF2 siRNA</t>
+  </si>
+  <si>
+    <t>PRJNA639359</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE152435</t>
+  </si>
+  <si>
+    <t>PRJNA639358</t>
+  </si>
+  <si>
+    <t>HeLa cells</t>
+  </si>
+  <si>
+    <t>Also looked at NBAS siRNA as activator of UPF1, looked at cyto and membrane</t>
+  </si>
+  <si>
+    <t>Also looked at NBAS siRNA as activator of UPF1</t>
   </si>
 </sst>
 </file>
@@ -3263,37 +3551,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E28C8A8-6FB1-4F0E-BBCF-A1462531D658}">
   <dimension ref="A1:AE80"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="32.5546875" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.44140625" customWidth="1"/>
-    <col min="10" max="12" width="20.88671875" customWidth="1"/>
-    <col min="13" max="13" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.88671875" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="32.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.42578125" customWidth="1"/>
+    <col min="10" max="12" width="20.85546875" customWidth="1"/>
+    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.85546875" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="20.88671875" customWidth="1"/>
-    <col min="28" max="28" width="23.88671875" customWidth="1"/>
-    <col min="29" max="29" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="20.88671875" customWidth="1"/>
+    <col min="17" max="17" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.85546875" customWidth="1"/>
+    <col min="28" max="28" width="23.85546875" customWidth="1"/>
+    <col min="29" max="29" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3385,7 +3673,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -3480,7 +3768,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -3575,7 +3863,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -3670,7 +3958,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
@@ -3765,7 +4053,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>28</v>
       </c>
@@ -3860,7 +4148,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -3955,7 +4243,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -4050,7 +4338,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>73</v>
       </c>
@@ -4145,7 +4433,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>73</v>
       </c>
@@ -4240,7 +4528,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>73</v>
       </c>
@@ -4335,7 +4623,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>73</v>
       </c>
@@ -4430,7 +4718,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>73</v>
       </c>
@@ -4525,7 +4813,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -4620,7 +4908,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>73</v>
       </c>
@@ -4715,7 +5003,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>73</v>
       </c>
@@ -4810,7 +5098,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>73</v>
       </c>
@@ -4905,7 +5193,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>73</v>
       </c>
@@ -5000,7 +5288,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>73</v>
       </c>
@@ -5095,7 +5383,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>73</v>
       </c>
@@ -5190,7 +5478,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>73</v>
       </c>
@@ -5285,7 +5573,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>73</v>
       </c>
@@ -5380,7 +5668,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>73</v>
       </c>
@@ -5475,7 +5763,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>73</v>
       </c>
@@ -5570,7 +5858,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>73</v>
       </c>
@@ -5665,7 +5953,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>73</v>
       </c>
@@ -5760,7 +6048,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>150</v>
       </c>
@@ -5852,7 +6140,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>150</v>
       </c>
@@ -5944,7 +6232,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>150</v>
       </c>
@@ -6036,7 +6324,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>150</v>
       </c>
@@ -6128,7 +6416,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>150</v>
       </c>
@@ -6220,7 +6508,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>150</v>
       </c>
@@ -6312,7 +6600,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>150</v>
       </c>
@@ -6404,7 +6692,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>150</v>
       </c>
@@ -6496,7 +6784,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>150</v>
       </c>
@@ -6588,7 +6876,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>150</v>
       </c>
@@ -6680,7 +6968,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>150</v>
       </c>
@@ -6772,7 +7060,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>150</v>
       </c>
@@ -6864,7 +7152,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>150</v>
       </c>
@@ -6956,7 +7244,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>150</v>
       </c>
@@ -7048,7 +7336,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>206</v>
       </c>
@@ -7140,7 +7428,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>206</v>
       </c>
@@ -7232,7 +7520,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>206</v>
       </c>
@@ -7324,7 +7612,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>206</v>
       </c>
@@ -7416,7 +7704,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>206</v>
       </c>
@@ -7508,7 +7796,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>206</v>
       </c>
@@ -7600,7 +7888,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>206</v>
       </c>
@@ -7692,7 +7980,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>206</v>
       </c>
@@ -7784,7 +8072,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>206</v>
       </c>
@@ -7876,7 +8164,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>206</v>
       </c>
@@ -7968,7 +8256,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>206</v>
       </c>
@@ -8060,7 +8348,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>206</v>
       </c>
@@ -8152,7 +8440,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>206</v>
       </c>
@@ -8244,7 +8532,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>206</v>
       </c>
@@ -8336,7 +8624,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>206</v>
       </c>
@@ -8428,7 +8716,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>206</v>
       </c>
@@ -8520,7 +8808,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>206</v>
       </c>
@@ -8612,7 +8900,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>206</v>
       </c>
@@ -8704,7 +8992,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>206</v>
       </c>
@@ -8796,7 +9084,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>206</v>
       </c>
@@ -8888,7 +9176,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>311</v>
       </c>
@@ -8983,7 +9271,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>311</v>
       </c>
@@ -9078,7 +9366,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>311</v>
       </c>
@@ -9173,7 +9461,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>311</v>
       </c>
@@ -9268,7 +9556,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>311</v>
       </c>
@@ -9363,7 +9651,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>311</v>
       </c>
@@ -9458,7 +9746,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>311</v>
       </c>
@@ -9553,7 +9841,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>311</v>
       </c>
@@ -9648,7 +9936,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>311</v>
       </c>
@@ -9743,7 +10031,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>311</v>
       </c>
@@ -9838,7 +10126,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>311</v>
       </c>
@@ -9933,7 +10221,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>311</v>
       </c>
@@ -10028,7 +10316,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>348</v>
       </c>
@@ -10120,7 +10408,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>348</v>
       </c>
@@ -10209,7 +10497,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>348</v>
       </c>
@@ -10298,7 +10586,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>348</v>
       </c>
@@ -10387,7 +10675,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>348</v>
       </c>
@@ -10479,7 +10767,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>348</v>
       </c>
@@ -10568,7 +10856,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>348</v>
       </c>
@@ -10657,7 +10945,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>348</v>
       </c>
@@ -10754,21 +11042,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1739B9-C94C-4465-8F8F-0F3F742A5026}">
   <dimension ref="A1:R87"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.6640625" customWidth="1"/>
-    <col min="5" max="5" width="44.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="79.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="18" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" customWidth="1"/>
+    <col min="5" max="5" width="44.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="79.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="18" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10824,7 +11112,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -10874,7 +11162,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -10918,7 +11206,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>150</v>
       </c>
@@ -10968,7 +11256,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>457</v>
       </c>
@@ -11018,7 +11306,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>461</v>
       </c>
@@ -11068,7 +11356,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>206</v>
       </c>
@@ -11121,7 +11409,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>311</v>
       </c>
@@ -11174,7 +11462,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>348</v>
       </c>
@@ -11221,7 +11509,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>469</v>
       </c>
@@ -11271,7 +11559,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>474</v>
       </c>
@@ -11318,7 +11606,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>478</v>
       </c>
@@ -11371,7 +11659,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>483</v>
       </c>
@@ -11415,7 +11703,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>487</v>
       </c>
@@ -11459,7 +11747,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>492</v>
       </c>
@@ -11503,7 +11791,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>497</v>
       </c>
@@ -11550,7 +11838,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>501</v>
       </c>
@@ -11597,7 +11885,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>505</v>
       </c>
@@ -11641,7 +11929,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>508</v>
       </c>
@@ -11688,7 +11976,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>513</v>
       </c>
@@ -11732,7 +12020,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>516</v>
       </c>
@@ -11776,7 +12064,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>519</v>
       </c>
@@ -11820,7 +12108,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>522</v>
       </c>
@@ -11864,7 +12152,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>524</v>
       </c>
@@ -11911,7 +12199,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>526</v>
       </c>
@@ -11955,7 +12243,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>529</v>
       </c>
@@ -12005,7 +12293,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>532</v>
       </c>
@@ -12046,7 +12334,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>535</v>
       </c>
@@ -12093,7 +12381,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>539</v>
       </c>
@@ -12137,7 +12425,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>542</v>
       </c>
@@ -12181,7 +12469,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>545</v>
       </c>
@@ -12225,7 +12513,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>548</v>
       </c>
@@ -12269,7 +12557,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>551</v>
       </c>
@@ -12280,7 +12568,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>554</v>
       </c>
@@ -12291,7 +12579,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>557</v>
       </c>
@@ -12302,7 +12590,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>560</v>
       </c>
@@ -12313,7 +12601,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>563</v>
       </c>
@@ -12324,7 +12612,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>565</v>
       </c>
@@ -12335,7 +12623,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>567</v>
       </c>
@@ -12346,7 +12634,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>570</v>
       </c>
@@ -12357,7 +12645,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>573</v>
       </c>
@@ -12368,7 +12656,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>576</v>
       </c>
@@ -12379,7 +12667,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>579</v>
       </c>
@@ -12390,7 +12678,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>582</v>
       </c>
@@ -12401,7 +12689,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>585</v>
       </c>
@@ -12412,7 +12700,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>588</v>
       </c>
@@ -12423,7 +12711,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>591</v>
       </c>
@@ -12434,7 +12722,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>594</v>
       </c>
@@ -12445,7 +12733,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>596</v>
       </c>
@@ -12456,7 +12744,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>598</v>
       </c>
@@ -12467,7 +12755,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>600</v>
       </c>
@@ -12478,7 +12766,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>602</v>
       </c>
@@ -12489,7 +12777,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>604</v>
       </c>
@@ -12500,7 +12788,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>606</v>
       </c>
@@ -12511,7 +12799,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>608</v>
       </c>
@@ -12522,7 +12810,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>610</v>
       </c>
@@ -12533,7 +12821,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>612</v>
       </c>
@@ -12550,7 +12838,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>617</v>
       </c>
@@ -12567,7 +12855,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
         <v>621</v>
       </c>
@@ -12584,7 +12872,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
         <v>625</v>
       </c>
@@ -12601,7 +12889,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
         <v>629</v>
       </c>
@@ -12618,7 +12906,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>633</v>
       </c>
@@ -12635,7 +12923,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
         <v>637</v>
       </c>
@@ -12652,7 +12940,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>641</v>
       </c>
@@ -12669,7 +12957,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
         <v>645</v>
       </c>
@@ -12686,7 +12974,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
         <v>649</v>
       </c>
@@ -12703,7 +12991,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
         <v>653</v>
       </c>
@@ -12720,7 +13008,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
         <v>657</v>
       </c>
@@ -12737,7 +13025,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
         <v>661</v>
       </c>
@@ -12754,7 +13042,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
         <v>665</v>
       </c>
@@ -12771,7 +13059,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
         <v>669</v>
       </c>
@@ -12788,7 +13076,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>669</v>
       </c>
@@ -12805,7 +13093,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
         <v>675</v>
       </c>
@@ -12822,7 +13110,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
         <v>679</v>
       </c>
@@ -12839,7 +13127,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
         <v>683</v>
       </c>
@@ -12856,7 +13144,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
         <v>683</v>
       </c>
@@ -12873,7 +13161,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
         <v>33</v>
       </c>
@@ -12890,7 +13178,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
         <v>33</v>
       </c>
@@ -12907,7 +13195,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
         <v>33</v>
       </c>
@@ -12924,7 +13212,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
         <v>33</v>
       </c>
@@ -12941,7 +13229,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
         <v>695</v>
       </c>
@@ -12958,7 +13246,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
         <v>695</v>
       </c>
@@ -12975,7 +13263,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
         <v>703</v>
       </c>
@@ -12992,7 +13280,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
         <v>708</v>
       </c>
@@ -13009,7 +13297,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
         <v>713</v>
       </c>
@@ -13033,21 +13321,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89C31724-8146-4D7C-A3D2-DC7D492096E6}">
-  <dimension ref="A1:L41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:R41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" customWidth="1"/>
+    <col min="12" max="15" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>718</v>
       </c>
@@ -13076,120 +13367,594 @@
         <v>726</v>
       </c>
       <c r="J1" t="s">
+        <v>769</v>
+      </c>
+      <c r="K1" t="s">
+        <v>783</v>
+      </c>
+      <c r="L1" t="s">
+        <v>784</v>
+      </c>
+      <c r="M1" t="s">
+        <v>777</v>
+      </c>
+      <c r="N1" t="s">
+        <v>770</v>
+      </c>
+      <c r="O1" t="s">
+        <v>789</v>
+      </c>
+      <c r="P1" t="s">
         <v>727</v>
       </c>
-      <c r="K1" t="s">
-        <v>728</v>
-      </c>
-      <c r="L1" t="s">
-        <v>764</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q1" t="s">
+        <v>763</v>
+      </c>
+      <c r="R1" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
+      <c r="B2" t="s">
+        <v>771</v>
+      </c>
+      <c r="C2" t="s">
+        <v>773</v>
+      </c>
+      <c r="E2" t="s">
+        <v>788</v>
+      </c>
+      <c r="F2" t="s">
+        <v>772</v>
+      </c>
       <c r="G2">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>736</v>
+      </c>
+      <c r="L2" t="s">
+        <v>776</v>
+      </c>
+      <c r="M2" t="s">
+        <v>801</v>
+      </c>
+      <c r="N2" t="s">
+        <v>782</v>
+      </c>
+      <c r="O2" t="s">
+        <v>790</v>
+      </c>
+      <c r="R2" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>73</v>
       </c>
+      <c r="B3" t="s">
+        <v>775</v>
+      </c>
+      <c r="C3" t="s">
+        <v>785</v>
+      </c>
+      <c r="E3" t="s">
+        <v>788</v>
+      </c>
+      <c r="F3" t="s">
+        <v>774</v>
+      </c>
       <c r="G3">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H3">
+        <v>12</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="K3" t="s">
+        <v>736</v>
+      </c>
+      <c r="L3" t="s">
+        <v>776</v>
+      </c>
+      <c r="M3" t="s">
+        <v>778</v>
+      </c>
+      <c r="N3" t="s">
+        <v>779</v>
+      </c>
+      <c r="O3" t="s">
+        <v>790</v>
+      </c>
+      <c r="R3" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>150</v>
       </c>
+      <c r="B4" t="s">
+        <v>787</v>
+      </c>
+      <c r="E4" t="s">
+        <v>796</v>
+      </c>
+      <c r="F4" t="s">
+        <v>786</v>
+      </c>
       <c r="G4">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <v>6</v>
+      </c>
+      <c r="I4">
+        <v>6</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4" t="s">
+        <v>424</v>
+      </c>
+      <c r="L4" t="s">
+        <v>793</v>
+      </c>
+      <c r="M4" t="s">
+        <v>778</v>
+      </c>
+      <c r="N4" t="s">
+        <v>792</v>
+      </c>
+      <c r="O4" t="s">
+        <v>791</v>
+      </c>
+      <c r="R4" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>206</v>
       </c>
+      <c r="B5" t="s">
+        <v>798</v>
+      </c>
+      <c r="E5" t="s">
+        <v>797</v>
+      </c>
+      <c r="F5" t="s">
+        <v>795</v>
+      </c>
       <c r="G5">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>8</v>
+      </c>
+      <c r="K5" t="s">
+        <v>834</v>
+      </c>
+      <c r="L5" t="s">
+        <v>802</v>
+      </c>
+      <c r="M5" t="s">
+        <v>778</v>
+      </c>
+      <c r="N5" t="s">
+        <v>799</v>
+      </c>
+      <c r="O5" t="s">
+        <v>800</v>
+      </c>
+      <c r="R5" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>311</v>
       </c>
+      <c r="B6" t="s">
+        <v>805</v>
+      </c>
+      <c r="C6" t="s">
+        <v>806</v>
+      </c>
+      <c r="E6" t="s">
+        <v>804</v>
+      </c>
+      <c r="F6" t="s">
+        <v>803</v>
+      </c>
       <c r="G6">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>819</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="K6" t="s">
+        <v>833</v>
+      </c>
+      <c r="M6" t="s">
+        <v>778</v>
+      </c>
+      <c r="N6" t="s">
+        <v>807</v>
+      </c>
+      <c r="O6" t="s">
+        <v>808</v>
+      </c>
+      <c r="R6" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>348</v>
       </c>
+      <c r="B7" t="s">
+        <v>812</v>
+      </c>
+      <c r="E7" t="s">
+        <v>813</v>
+      </c>
+      <c r="F7" t="s">
+        <v>811</v>
+      </c>
       <c r="G7">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>4</v>
+      </c>
+      <c r="K7" t="s">
+        <v>817</v>
+      </c>
+      <c r="L7" t="s">
+        <v>816</v>
+      </c>
+      <c r="M7" t="s">
+        <v>778</v>
+      </c>
+      <c r="N7" t="s">
+        <v>814</v>
+      </c>
+      <c r="O7" t="s">
+        <v>815</v>
+      </c>
+      <c r="R7" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>469</v>
       </c>
+      <c r="B8" t="s">
+        <v>823</v>
+      </c>
+      <c r="C8" t="s">
+        <v>824</v>
+      </c>
+      <c r="E8" t="s">
+        <v>820</v>
+      </c>
+      <c r="F8" t="s">
+        <v>821</v>
+      </c>
       <c r="G8">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H8">
+        <v>6</v>
+      </c>
+      <c r="I8">
+        <v>6</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8" t="s">
+        <v>736</v>
+      </c>
+      <c r="L8" t="s">
+        <v>827</v>
+      </c>
+      <c r="M8" t="s">
+        <v>778</v>
+      </c>
+      <c r="N8" t="s">
+        <v>825</v>
+      </c>
+      <c r="O8" t="s">
+        <v>822</v>
+      </c>
+      <c r="R8" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>478</v>
       </c>
+      <c r="B9" t="s">
+        <v>830</v>
+      </c>
+      <c r="E9" t="s">
+        <v>829</v>
+      </c>
+      <c r="F9" t="s">
+        <v>828</v>
+      </c>
       <c r="G9">
         <v>41</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H9">
+        <v>12</v>
+      </c>
+      <c r="I9">
+        <v>29</v>
+      </c>
+      <c r="K9" t="s">
+        <v>415</v>
+      </c>
+      <c r="L9" t="s">
+        <v>835</v>
+      </c>
+      <c r="M9" t="s">
+        <v>778</v>
+      </c>
+      <c r="N9" t="s">
+        <v>839</v>
+      </c>
+      <c r="O9" t="s">
+        <v>832</v>
+      </c>
+      <c r="R9" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>483</v>
       </c>
+      <c r="B10" t="s">
+        <v>838</v>
+      </c>
+      <c r="E10" t="s">
+        <v>837</v>
+      </c>
+      <c r="F10" t="s">
+        <v>836</v>
+      </c>
       <c r="G10">
         <v>143</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H10">
+        <v>71</v>
+      </c>
+      <c r="I10">
+        <v>72</v>
+      </c>
+      <c r="K10" t="s">
+        <v>817</v>
+      </c>
+      <c r="M10" t="s">
+        <v>778</v>
+      </c>
+      <c r="N10" t="s">
+        <v>840</v>
+      </c>
+      <c r="O10" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>529</v>
       </c>
+      <c r="B11" t="s">
+        <v>846</v>
+      </c>
+      <c r="E11" t="s">
+        <v>843</v>
+      </c>
+      <c r="F11" t="s">
+        <v>842</v>
+      </c>
       <c r="G11">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H11">
+        <v>6</v>
+      </c>
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="K11" t="s">
+        <v>847</v>
+      </c>
+      <c r="M11" t="s">
+        <v>778</v>
+      </c>
+      <c r="N11" t="s">
+        <v>845</v>
+      </c>
+      <c r="O11" t="s">
+        <v>844</v>
+      </c>
+      <c r="R11" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>612</v>
       </c>
+      <c r="B12" t="s">
+        <v>851</v>
+      </c>
+      <c r="C12" t="s">
+        <v>613</v>
+      </c>
+      <c r="E12" t="s">
+        <v>849</v>
+      </c>
+      <c r="F12" t="s">
+        <v>850</v>
+      </c>
       <c r="G12">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H12">
+        <v>3</v>
+      </c>
+      <c r="I12">
+        <v>3</v>
+      </c>
+      <c r="J12">
+        <v>6</v>
+      </c>
+      <c r="K12" t="s">
+        <v>424</v>
+      </c>
+      <c r="L12" t="s">
+        <v>853</v>
+      </c>
+      <c r="M12" t="s">
+        <v>778</v>
+      </c>
+      <c r="N12" t="s">
+        <v>852</v>
+      </c>
+      <c r="O12" t="s">
+        <v>854</v>
+      </c>
+      <c r="R12" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>617</v>
       </c>
+      <c r="B13" t="s">
+        <v>860</v>
+      </c>
+      <c r="C13" t="s">
+        <v>618</v>
+      </c>
+      <c r="E13" t="s">
+        <v>857</v>
+      </c>
+      <c r="F13" t="s">
+        <v>856</v>
+      </c>
       <c r="G13">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <v>6</v>
+      </c>
+      <c r="I13">
+        <v>6</v>
+      </c>
+      <c r="J13">
+        <v>12</v>
+      </c>
+      <c r="K13" t="s">
+        <v>859</v>
+      </c>
+      <c r="M13" t="s">
+        <v>778</v>
+      </c>
+      <c r="N13" t="s">
+        <v>858</v>
+      </c>
+      <c r="O13" t="s">
+        <v>863</v>
+      </c>
+      <c r="R13" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>621</v>
       </c>
+      <c r="B14" t="s">
+        <v>862</v>
+      </c>
+      <c r="C14" t="s">
+        <v>622</v>
+      </c>
+      <c r="E14" t="s">
+        <v>857</v>
+      </c>
+      <c r="F14" t="s">
+        <v>861</v>
+      </c>
       <c r="G14">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H14">
+        <v>5</v>
+      </c>
+      <c r="I14">
+        <v>5</v>
+      </c>
+      <c r="J14">
+        <v>5</v>
+      </c>
+      <c r="K14" t="s">
+        <v>424</v>
+      </c>
+      <c r="M14" t="s">
+        <v>778</v>
+      </c>
+      <c r="N14" t="s">
+        <v>858</v>
+      </c>
+      <c r="O14" t="s">
+        <v>863</v>
+      </c>
+      <c r="R14" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>625</v>
       </c>
@@ -13197,7 +13962,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>629</v>
       </c>
@@ -13205,7 +13970,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>633</v>
       </c>
@@ -13213,7 +13978,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>637</v>
       </c>
@@ -13221,368 +13986,368 @@
         <v>166</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
         <v>641</v>
       </c>
       <c r="F19" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G19">
         <v>24</v>
       </c>
-      <c r="J19" t="s">
-        <v>748</v>
-      </c>
       <c r="L19" t="s">
         <v>747</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q19" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
         <v>645</v>
       </c>
       <c r="F20" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="G20">
         <v>18</v>
       </c>
-      <c r="J20" t="s">
-        <v>746</v>
-      </c>
       <c r="L20" t="s">
         <v>745</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q20" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
         <v>649</v>
       </c>
       <c r="F21" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="G21">
         <v>15</v>
       </c>
-      <c r="J21" t="s">
-        <v>751</v>
-      </c>
       <c r="L21" t="s">
         <v>750</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q21" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
         <v>653</v>
       </c>
       <c r="F22" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="G22">
         <v>24</v>
       </c>
-      <c r="J22" t="s">
-        <v>754</v>
-      </c>
       <c r="L22" t="s">
         <v>753</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q22" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
         <v>657</v>
       </c>
       <c r="F23" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G23">
         <v>27</v>
       </c>
-      <c r="J23" t="s">
-        <v>757</v>
-      </c>
       <c r="L23" t="s">
         <v>756</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q23" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
         <v>661</v>
       </c>
       <c r="F24" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G24">
         <v>24</v>
       </c>
-      <c r="J24" t="s">
-        <v>754</v>
-      </c>
       <c r="L24" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+        <v>753</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
         <v>665</v>
       </c>
       <c r="F25" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G25">
         <v>9</v>
       </c>
-      <c r="J25" t="s">
-        <v>754</v>
-      </c>
       <c r="L25" t="s">
-        <v>761</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+        <v>753</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
         <v>669</v>
       </c>
       <c r="F26" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G26">
         <v>18</v>
       </c>
-      <c r="J26" t="s">
-        <v>763</v>
-      </c>
-      <c r="L26" s="10" t="s">
+      <c r="L26" t="s">
+        <v>762</v>
+      </c>
+      <c r="Q26" s="10" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
         <v>669</v>
       </c>
       <c r="F27" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G27">
         <v>18</v>
       </c>
-      <c r="J27" t="s">
-        <v>763</v>
-      </c>
-      <c r="L27" s="10" t="s">
+      <c r="L27" t="s">
+        <v>762</v>
+      </c>
+      <c r="Q27" s="10" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
         <v>675</v>
       </c>
       <c r="F28" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="G28">
         <v>21</v>
       </c>
-      <c r="J28" t="s">
-        <v>757</v>
-      </c>
       <c r="L28" t="s">
         <v>756</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q28" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="F29" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="G29">
         <v>27</v>
       </c>
-      <c r="J29" t="s">
-        <v>737</v>
-      </c>
       <c r="L29" t="s">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+        <v>736</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
         <v>679</v>
       </c>
       <c r="F30" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="G30">
         <v>36</v>
       </c>
-      <c r="J30" t="s">
+      <c r="L30" t="s">
+        <v>736</v>
+      </c>
+      <c r="Q30" t="s">
         <v>737</v>
       </c>
-      <c r="L30" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
         <v>683</v>
       </c>
       <c r="F31" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="G31">
         <v>12</v>
       </c>
-      <c r="J31" t="s">
-        <v>767</v>
-      </c>
       <c r="L31" t="s">
+        <v>766</v>
+      </c>
+      <c r="Q31" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
         <v>683</v>
       </c>
       <c r="F32" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="G32">
         <v>12</v>
       </c>
-      <c r="J32" t="s">
-        <v>767</v>
-      </c>
       <c r="L32" t="s">
+        <v>766</v>
+      </c>
+      <c r="Q32" t="s">
         <v>687</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
         <v>695</v>
       </c>
       <c r="F33" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="G33">
         <v>8</v>
       </c>
-      <c r="J33" t="s">
-        <v>757</v>
-      </c>
-      <c r="K33" t="s">
+      <c r="L33" t="s">
+        <v>756</v>
+      </c>
+      <c r="P33" t="s">
         <v>697</v>
       </c>
-      <c r="L33" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q33" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
         <v>695</v>
       </c>
       <c r="F34" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="G34">
         <v>8</v>
       </c>
-      <c r="J34" t="s">
-        <v>757</v>
-      </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
+        <v>756</v>
+      </c>
+      <c r="P34" t="s">
         <v>700</v>
       </c>
-      <c r="L34" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q34" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D35" t="s">
         <v>703</v>
       </c>
       <c r="F35" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="G35">
         <v>6</v>
       </c>
-      <c r="J35" t="s">
-        <v>754</v>
-      </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
+        <v>753</v>
+      </c>
+      <c r="P35" t="s">
         <v>705</v>
       </c>
-      <c r="L35" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="Q35" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>708</v>
       </c>
       <c r="G36">
         <v>6</v>
       </c>
-      <c r="K36" t="s">
+      <c r="P36" t="s">
         <v>710</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>713</v>
       </c>
       <c r="G37">
         <v>36</v>
       </c>
-      <c r="K37" t="s">
+      <c r="P37" t="s">
         <v>715</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
+        <v>728</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="L38" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
         <v>729</v>
       </c>
-      <c r="G38">
-        <v>1</v>
-      </c>
-      <c r="J38" t="s">
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="L39" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C39" t="s">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
         <v>730</v>
       </c>
-      <c r="G39">
-        <v>1</v>
-      </c>
-      <c r="J39" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C40" t="s">
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="L40" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
         <v>731</v>
       </c>
-      <c r="G40">
-        <v>1</v>
-      </c>
-      <c r="J40" t="s">
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="L41" t="s">
         <v>733</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C41" t="s">
-        <v>732</v>
-      </c>
-      <c r="G41">
-        <v>1</v>
-      </c>
-      <c r="J41" t="s">
-        <v>734</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add additiona dataset meta info
</commit_message>
<xml_diff>
--- a/data/NMD_Perturbation_TopStudySamples_20260712.xlsx
+++ b/data/NMD_Perturbation_TopStudySamples_20260712.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://moffitt-my.sharepoint.com/personal/alyssa_obermayer_moffitt_org/Documents/Documents/Projects/Active/NMD_Perturbation/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\aobermayer4\Projects\active\Public_NMD_Perturbation_Data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="13_ncr:1_{5A1180FC-E05E-412E-A9C8-872707654177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBB80609-CB8B-4057-A715-107CBCEA5C66}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2586E139-F2AC-480F-9FE3-F3A5C02AEE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
   </bookViews>
   <sheets>
     <sheet name="NMD_Perturbation_TopStudySample" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2357" uniqueCount="866">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2395" uniqueCount="894">
   <si>
     <t>GSE_ID</t>
   </si>
@@ -2620,13 +2620,97 @@
   </si>
   <si>
     <t>Also looked at NBAS siRNA as activator of UPF1</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE176197</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9108617/</t>
+  </si>
+  <si>
+    <t>PRJNA735254</t>
+  </si>
+  <si>
+    <t>Flp-In T-REx-293 cells</t>
+  </si>
+  <si>
+    <t>a specialized mammalian host line used for generating stable, isogenic cell lines with tightly regulated, inducible protein expression. They are ideal for high-level expression and functional studies of toxic or tightly controlled genes. [1, 2, 3, 4, 5]</t>
+  </si>
+  <si>
+    <t>GSE134059</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE134059</t>
+  </si>
+  <si>
+    <t>PRJNA553576</t>
+  </si>
+  <si>
+    <t>SRP213944</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE162699</t>
+  </si>
+  <si>
+    <t>PRJNA682628</t>
+  </si>
+  <si>
+    <t>SRP295982</t>
+  </si>
+  <si>
+    <t>GSE162699</t>
+  </si>
+  <si>
+    <t>GSE59884</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE59884</t>
+  </si>
+  <si>
+    <t>PRJNA256984</t>
+  </si>
+  <si>
+    <t>SRP045065</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC4764554/</t>
+  </si>
+  <si>
+    <t>HEK-293T</t>
+  </si>
+  <si>
+    <t>non-targeting control siRNA or UPF1LL-specific siRNA were treated with vehicle control, puromycin, or thapsigargin</t>
+  </si>
+  <si>
+    <t>UPF1LL siRNA</t>
+  </si>
+  <si>
+    <t>HEK-293 Trex cells</t>
+  </si>
+  <si>
+    <t>overexpression of CLIP-tagged UPF1 isoforms 1 and 2 or GFP</t>
+  </si>
+  <si>
+    <t>UPF1LL/SL Overexpression</t>
+  </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9108617/#embj2021108898-sec-0021</t>
+  </si>
+  <si>
+    <t>RIPseq, RNAseq</t>
+  </si>
+  <si>
+    <t>RNAseq</t>
+  </si>
+  <si>
+    <t>RIPseq</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2770,6 +2854,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3114,7 +3206,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="43">
+  <cellStyleXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -3158,8 +3250,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -3174,8 +3267,10 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="43"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="43">
+  <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -3209,6 +3304,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="43" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -3551,37 +3647,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E28C8A8-6FB1-4F0E-BBCF-A1462531D658}">
   <dimension ref="A1:AE80"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="32.5703125" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.42578125" customWidth="1"/>
-    <col min="10" max="12" width="20.85546875" customWidth="1"/>
-    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="32.5546875" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.44140625" customWidth="1"/>
+    <col min="10" max="12" width="20.88671875" customWidth="1"/>
+    <col min="13" max="13" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.88671875" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="20.85546875" customWidth="1"/>
-    <col min="28" max="28" width="23.85546875" customWidth="1"/>
-    <col min="29" max="29" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="20.85546875" customWidth="1"/>
+    <col min="17" max="17" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.88671875" customWidth="1"/>
+    <col min="28" max="28" width="23.88671875" customWidth="1"/>
+    <col min="29" max="29" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="20.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3673,7 +3769,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -3768,7 +3864,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -3863,7 +3959,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -3958,7 +4054,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
@@ -4053,7 +4149,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>28</v>
       </c>
@@ -4148,7 +4244,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -4243,7 +4339,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -4338,7 +4434,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>73</v>
       </c>
@@ -4433,7 +4529,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>73</v>
       </c>
@@ -4528,7 +4624,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>73</v>
       </c>
@@ -4623,7 +4719,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>73</v>
       </c>
@@ -4718,7 +4814,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>73</v>
       </c>
@@ -4813,7 +4909,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -4908,7 +5004,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>73</v>
       </c>
@@ -5003,7 +5099,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>73</v>
       </c>
@@ -5098,7 +5194,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5193,7 +5289,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>73</v>
       </c>
@@ -5288,7 +5384,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>73</v>
       </c>
@@ -5383,7 +5479,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>73</v>
       </c>
@@ -5478,7 +5574,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>73</v>
       </c>
@@ -5573,7 +5669,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>73</v>
       </c>
@@ -5668,7 +5764,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>73</v>
       </c>
@@ -5763,7 +5859,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>73</v>
       </c>
@@ -5858,7 +5954,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>73</v>
       </c>
@@ -5953,7 +6049,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>73</v>
       </c>
@@ -6048,7 +6144,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>150</v>
       </c>
@@ -6140,7 +6236,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>150</v>
       </c>
@@ -6232,7 +6328,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>150</v>
       </c>
@@ -6324,7 +6420,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>150</v>
       </c>
@@ -6416,7 +6512,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>150</v>
       </c>
@@ -6508,7 +6604,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>150</v>
       </c>
@@ -6600,7 +6696,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>150</v>
       </c>
@@ -6692,7 +6788,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>150</v>
       </c>
@@ -6784,7 +6880,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>150</v>
       </c>
@@ -6876,7 +6972,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>150</v>
       </c>
@@ -6968,7 +7064,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>150</v>
       </c>
@@ -7060,7 +7156,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>150</v>
       </c>
@@ -7152,7 +7248,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>150</v>
       </c>
@@ -7244,7 +7340,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>150</v>
       </c>
@@ -7336,7 +7432,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>206</v>
       </c>
@@ -7428,7 +7524,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>206</v>
       </c>
@@ -7520,7 +7616,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>206</v>
       </c>
@@ -7612,7 +7708,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>206</v>
       </c>
@@ -7704,7 +7800,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>206</v>
       </c>
@@ -7796,7 +7892,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>206</v>
       </c>
@@ -7888,7 +7984,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>206</v>
       </c>
@@ -7980,7 +8076,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>206</v>
       </c>
@@ -8072,7 +8168,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>206</v>
       </c>
@@ -8164,7 +8260,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>206</v>
       </c>
@@ -8256,7 +8352,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>206</v>
       </c>
@@ -8348,7 +8444,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>206</v>
       </c>
@@ -8440,7 +8536,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>206</v>
       </c>
@@ -8532,7 +8628,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>206</v>
       </c>
@@ -8624,7 +8720,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>206</v>
       </c>
@@ -8716,7 +8812,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>206</v>
       </c>
@@ -8808,7 +8904,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>206</v>
       </c>
@@ -8900,7 +8996,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>206</v>
       </c>
@@ -8992,7 +9088,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>206</v>
       </c>
@@ -9084,7 +9180,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>206</v>
       </c>
@@ -9176,7 +9272,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>311</v>
       </c>
@@ -9271,7 +9367,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>311</v>
       </c>
@@ -9366,7 +9462,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>311</v>
       </c>
@@ -9461,7 +9557,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>311</v>
       </c>
@@ -9556,7 +9652,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>311</v>
       </c>
@@ -9651,7 +9747,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>311</v>
       </c>
@@ -9746,7 +9842,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>311</v>
       </c>
@@ -9841,7 +9937,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>311</v>
       </c>
@@ -9936,7 +10032,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>311</v>
       </c>
@@ -10031,7 +10127,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>311</v>
       </c>
@@ -10126,7 +10222,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>311</v>
       </c>
@@ -10221,7 +10317,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>311</v>
       </c>
@@ -10316,7 +10412,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>348</v>
       </c>
@@ -10408,7 +10504,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>348</v>
       </c>
@@ -10497,7 +10593,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>348</v>
       </c>
@@ -10586,7 +10682,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>348</v>
       </c>
@@ -10675,7 +10771,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>348</v>
       </c>
@@ -10767,7 +10863,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>348</v>
       </c>
@@ -10856,7 +10952,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>348</v>
       </c>
@@ -10945,7 +11041,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>348</v>
       </c>
@@ -11042,21 +11138,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1739B9-C94C-4465-8F8F-0F3F742A5026}">
   <dimension ref="A1:R87"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" customWidth="1"/>
-    <col min="5" max="5" width="44.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="79.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="18" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.6640625" customWidth="1"/>
+    <col min="5" max="5" width="44.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="79.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="18" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11112,7 +11208,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -11162,7 +11258,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -11206,7 +11302,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>150</v>
       </c>
@@ -11256,7 +11352,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>457</v>
       </c>
@@ -11306,7 +11402,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>461</v>
       </c>
@@ -11356,7 +11452,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>206</v>
       </c>
@@ -11409,7 +11505,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>311</v>
       </c>
@@ -11462,7 +11558,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>348</v>
       </c>
@@ -11509,7 +11605,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>469</v>
       </c>
@@ -11559,7 +11655,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>474</v>
       </c>
@@ -11606,7 +11702,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>478</v>
       </c>
@@ -11659,7 +11755,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>483</v>
       </c>
@@ -11703,7 +11799,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>487</v>
       </c>
@@ -11747,7 +11843,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>492</v>
       </c>
@@ -11791,7 +11887,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>497</v>
       </c>
@@ -11838,7 +11934,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>501</v>
       </c>
@@ -11885,7 +11981,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>505</v>
       </c>
@@ -11929,7 +12025,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>508</v>
       </c>
@@ -11976,7 +12072,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>513</v>
       </c>
@@ -12020,7 +12116,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>516</v>
       </c>
@@ -12064,7 +12160,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>519</v>
       </c>
@@ -12108,7 +12204,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>522</v>
       </c>
@@ -12152,7 +12248,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>524</v>
       </c>
@@ -12199,7 +12295,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>526</v>
       </c>
@@ -12243,7 +12339,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>529</v>
       </c>
@@ -12293,7 +12389,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>532</v>
       </c>
@@ -12334,7 +12430,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>535</v>
       </c>
@@ -12381,7 +12477,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>539</v>
       </c>
@@ -12425,7 +12521,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>542</v>
       </c>
@@ -12469,7 +12565,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>545</v>
       </c>
@@ -12513,7 +12609,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>548</v>
       </c>
@@ -12557,7 +12653,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>551</v>
       </c>
@@ -12568,7 +12664,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>554</v>
       </c>
@@ -12579,7 +12675,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>557</v>
       </c>
@@ -12590,7 +12686,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>560</v>
       </c>
@@ -12601,7 +12697,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>563</v>
       </c>
@@ -12612,7 +12708,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>565</v>
       </c>
@@ -12623,7 +12719,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>567</v>
       </c>
@@ -12634,7 +12730,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>570</v>
       </c>
@@ -12645,7 +12741,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>573</v>
       </c>
@@ -12656,7 +12752,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>576</v>
       </c>
@@ -12667,7 +12763,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>579</v>
       </c>
@@ -12678,7 +12774,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>582</v>
       </c>
@@ -12689,7 +12785,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>585</v>
       </c>
@@ -12700,7 +12796,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>588</v>
       </c>
@@ -12711,7 +12807,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>591</v>
       </c>
@@ -12722,7 +12818,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>594</v>
       </c>
@@ -12733,7 +12829,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>596</v>
       </c>
@@ -12744,7 +12840,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>598</v>
       </c>
@@ -12755,7 +12851,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>600</v>
       </c>
@@ -12766,7 +12862,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>602</v>
       </c>
@@ -12777,7 +12873,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>604</v>
       </c>
@@ -12788,7 +12884,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>606</v>
       </c>
@@ -12799,7 +12895,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>608</v>
       </c>
@@ -12810,7 +12906,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>610</v>
       </c>
@@ -12821,7 +12917,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
         <v>612</v>
       </c>
@@ -12838,7 +12934,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
         <v>617</v>
       </c>
@@ -12855,7 +12951,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
         <v>621</v>
       </c>
@@ -12872,7 +12968,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="9" t="s">
         <v>625</v>
       </c>
@@ -12889,7 +12985,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="10" t="s">
         <v>629</v>
       </c>
@@ -12906,7 +13002,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
         <v>633</v>
       </c>
@@ -12923,7 +13019,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="10" t="s">
         <v>637</v>
       </c>
@@ -12940,7 +13036,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
         <v>641</v>
       </c>
@@ -12957,7 +13053,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="10" t="s">
         <v>645</v>
       </c>
@@ -12974,7 +13070,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="10" t="s">
         <v>649</v>
       </c>
@@ -12991,7 +13087,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="10" t="s">
         <v>653</v>
       </c>
@@ -13008,7 +13104,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="10" t="s">
         <v>657</v>
       </c>
@@ -13025,7 +13121,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
         <v>661</v>
       </c>
@@ -13042,7 +13138,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="10" t="s">
         <v>665</v>
       </c>
@@ -13059,7 +13155,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="10" t="s">
         <v>669</v>
       </c>
@@ -13076,7 +13172,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="10" t="s">
         <v>669</v>
       </c>
@@ -13093,7 +13189,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="10" t="s">
         <v>675</v>
       </c>
@@ -13110,7 +13206,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="10" t="s">
         <v>679</v>
       </c>
@@ -13127,7 +13223,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="10" t="s">
         <v>683</v>
       </c>
@@ -13144,7 +13240,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
         <v>683</v>
       </c>
@@ -13161,7 +13257,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="10" t="s">
         <v>33</v>
       </c>
@@ -13178,7 +13274,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="10" t="s">
         <v>33</v>
       </c>
@@ -13195,7 +13291,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="10" t="s">
         <v>33</v>
       </c>
@@ -13212,7 +13308,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="10" t="s">
         <v>33</v>
       </c>
@@ -13229,7 +13325,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="10" t="s">
         <v>695</v>
       </c>
@@ -13246,7 +13342,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="10" t="s">
         <v>695</v>
       </c>
@@ -13263,7 +13359,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="10" t="s">
         <v>703</v>
       </c>
@@ -13280,7 +13376,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="10" t="s">
         <v>708</v>
       </c>
@@ -13297,7 +13393,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="10" t="s">
         <v>713</v>
       </c>
@@ -13321,24 +13417,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89C31724-8146-4D7C-A3D2-DC7D492096E6}">
-  <dimension ref="A1:R41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R44"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.44140625" customWidth="1"/>
+    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" customWidth="1"/>
-    <col min="12" max="15" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" customWidth="1"/>
+    <col min="12" max="15" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>718</v>
       </c>
@@ -13394,7 +13490,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -13441,7 +13537,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -13485,7 +13581,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>150</v>
       </c>
@@ -13529,7 +13625,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>206</v>
       </c>
@@ -13573,7 +13669,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>311</v>
       </c>
@@ -13614,7 +13710,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>348</v>
       </c>
@@ -13658,7 +13754,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>469</v>
       </c>
@@ -13705,7 +13801,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>478</v>
       </c>
@@ -13746,7 +13842,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>483</v>
       </c>
@@ -13781,7 +13877,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>529</v>
       </c>
@@ -13819,7 +13915,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>612</v>
       </c>
@@ -13866,7 +13962,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>617</v>
       </c>
@@ -13910,7 +14006,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>621</v>
       </c>
@@ -13954,403 +14050,565 @@
         <v>865</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>625</v>
       </c>
+      <c r="B15" t="s">
+        <v>868</v>
+      </c>
+      <c r="C15" t="s">
+        <v>626</v>
+      </c>
+      <c r="E15" t="s">
+        <v>867</v>
+      </c>
+      <c r="F15" t="s">
+        <v>866</v>
+      </c>
       <c r="G15">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>3</v>
+      </c>
+      <c r="K15" t="s">
+        <v>424</v>
+      </c>
+      <c r="M15" t="s">
+        <v>778</v>
+      </c>
+      <c r="N15" t="s">
+        <v>869</v>
+      </c>
+      <c r="O15" t="s">
+        <v>870</v>
+      </c>
+      <c r="P15" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>871</v>
+      </c>
+      <c r="B16" t="s">
+        <v>873</v>
+      </c>
+      <c r="C16" t="s">
+        <v>874</v>
+      </c>
+      <c r="E16" t="s">
+        <v>890</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>872</v>
+      </c>
+      <c r="G16">
+        <v>15</v>
+      </c>
+      <c r="H16">
+        <v>12</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="K16" t="s">
+        <v>889</v>
+      </c>
+      <c r="L16" t="s">
+        <v>888</v>
+      </c>
+      <c r="M16" t="s">
+        <v>778</v>
+      </c>
+      <c r="N16" t="s">
+        <v>887</v>
+      </c>
+      <c r="P16" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>878</v>
+      </c>
+      <c r="B17" t="s">
+        <v>876</v>
+      </c>
+      <c r="C17" t="s">
+        <v>877</v>
+      </c>
+      <c r="E17" t="s">
+        <v>867</v>
+      </c>
+      <c r="F17" t="s">
+        <v>875</v>
+      </c>
+      <c r="G17">
+        <v>48</v>
+      </c>
+      <c r="H17">
+        <v>9</v>
+      </c>
+      <c r="I17">
+        <v>9</v>
+      </c>
+      <c r="J17">
+        <v>30</v>
+      </c>
+      <c r="K17" t="s">
+        <v>886</v>
+      </c>
+      <c r="L17" t="s">
+        <v>885</v>
+      </c>
+      <c r="M17" t="s">
+        <v>778</v>
+      </c>
+      <c r="N17" t="s">
+        <v>852</v>
+      </c>
+      <c r="P17" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>879</v>
+      </c>
+      <c r="B18" t="s">
+        <v>881</v>
+      </c>
+      <c r="C18" t="s">
+        <v>882</v>
+      </c>
+      <c r="E18" t="s">
+        <v>883</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>880</v>
+      </c>
+      <c r="G18">
+        <v>8</v>
+      </c>
+      <c r="H18">
+        <v>2</v>
+      </c>
+      <c r="I18">
+        <v>2</v>
+      </c>
+      <c r="J18">
+        <v>4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>424</v>
+      </c>
+      <c r="M18" t="s">
+        <v>778</v>
+      </c>
+      <c r="N18" t="s">
+        <v>884</v>
+      </c>
+      <c r="P18" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>629</v>
       </c>
-      <c r="G16">
+      <c r="G19">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>633</v>
       </c>
-      <c r="G17">
+      <c r="G20">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>637</v>
       </c>
-      <c r="G18">
+      <c r="G21">
         <v>166</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D19" t="s">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D22" t="s">
         <v>641</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F22" t="s">
         <v>742</v>
-      </c>
-      <c r="G19">
-        <v>24</v>
-      </c>
-      <c r="L19" t="s">
-        <v>747</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D20" t="s">
-        <v>645</v>
-      </c>
-      <c r="F20" t="s">
-        <v>743</v>
-      </c>
-      <c r="G20">
-        <v>18</v>
-      </c>
-      <c r="L20" t="s">
-        <v>745</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
-        <v>649</v>
-      </c>
-      <c r="F21" t="s">
-        <v>748</v>
-      </c>
-      <c r="G21">
-        <v>15</v>
-      </c>
-      <c r="L21" t="s">
-        <v>750</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>749</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>653</v>
-      </c>
-      <c r="F22" t="s">
-        <v>751</v>
       </c>
       <c r="G22">
         <v>24</v>
       </c>
       <c r="L22" t="s">
-        <v>753</v>
+        <v>747</v>
       </c>
       <c r="Q22" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="D23" t="s">
-        <v>657</v>
+        <v>645</v>
       </c>
       <c r="F23" t="s">
-        <v>754</v>
+        <v>743</v>
       </c>
       <c r="G23">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="L23" t="s">
-        <v>756</v>
+        <v>745</v>
       </c>
       <c r="Q23" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="D24" t="s">
-        <v>661</v>
+        <v>649</v>
       </c>
       <c r="F24" t="s">
-        <v>757</v>
+        <v>748</v>
       </c>
       <c r="G24">
+        <v>15</v>
+      </c>
+      <c r="L24" t="s">
+        <v>750</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D25" t="s">
+        <v>653</v>
+      </c>
+      <c r="F25" t="s">
+        <v>751</v>
+      </c>
+      <c r="G25">
         <v>24</v>
-      </c>
-      <c r="L24" t="s">
-        <v>753</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D25" t="s">
-        <v>665</v>
-      </c>
-      <c r="F25" t="s">
-        <v>759</v>
-      </c>
-      <c r="G25">
-        <v>9</v>
       </c>
       <c r="L25" t="s">
         <v>753</v>
       </c>
       <c r="Q25" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D26" t="s">
+        <v>657</v>
+      </c>
+      <c r="F26" t="s">
+        <v>754</v>
+      </c>
+      <c r="G26">
+        <v>27</v>
+      </c>
+      <c r="L26" t="s">
+        <v>756</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D27" t="s">
+        <v>661</v>
+      </c>
+      <c r="F27" t="s">
+        <v>757</v>
+      </c>
+      <c r="G27">
+        <v>24</v>
+      </c>
+      <c r="L27" t="s">
+        <v>753</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D28" t="s">
+        <v>665</v>
+      </c>
+      <c r="F28" t="s">
+        <v>759</v>
+      </c>
+      <c r="G28">
+        <v>9</v>
+      </c>
+      <c r="L28" t="s">
+        <v>753</v>
+      </c>
+      <c r="Q28" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D26" t="s">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D29" t="s">
         <v>669</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F29" t="s">
         <v>761</v>
       </c>
-      <c r="G26">
+      <c r="G29">
         <v>18</v>
       </c>
-      <c r="L26" t="s">
+      <c r="L29" t="s">
         <v>762</v>
       </c>
-      <c r="Q26" s="10" t="s">
+      <c r="Q29" s="10" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D27" t="s">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D30" t="s">
         <v>669</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F30" t="s">
         <v>761</v>
       </c>
-      <c r="G27">
+      <c r="G30">
         <v>18</v>
       </c>
-      <c r="L27" t="s">
+      <c r="L30" t="s">
         <v>762</v>
       </c>
-      <c r="Q27" s="10" t="s">
+      <c r="Q30" s="10" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D31" t="s">
         <v>675</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F31" t="s">
         <v>764</v>
       </c>
-      <c r="G28">
+      <c r="G31">
         <v>21</v>
       </c>
-      <c r="L28" t="s">
+      <c r="L31" t="s">
         <v>756</v>
       </c>
-      <c r="Q28" t="s">
+      <c r="Q31" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D29" t="s">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D32" t="s">
         <v>738</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F32" t="s">
         <v>740</v>
       </c>
-      <c r="G29">
+      <c r="G32">
         <v>27</v>
       </c>
-      <c r="L29" t="s">
+      <c r="L32" t="s">
         <v>736</v>
       </c>
-      <c r="Q29" t="s">
+      <c r="Q32" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D30" t="s">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D33" t="s">
         <v>679</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F33" t="s">
         <v>741</v>
       </c>
-      <c r="G30">
+      <c r="G33">
         <v>36</v>
       </c>
-      <c r="L30" t="s">
+      <c r="L33" t="s">
         <v>736</v>
       </c>
-      <c r="Q30" t="s">
+      <c r="Q33" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D31" t="s">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D34" t="s">
         <v>683</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F34" t="s">
         <v>765</v>
       </c>
-      <c r="G31">
+      <c r="G34">
         <v>12</v>
       </c>
-      <c r="L31" t="s">
+      <c r="L34" t="s">
         <v>766</v>
       </c>
-      <c r="Q31" t="s">
+      <c r="Q34" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D32" t="s">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D35" t="s">
         <v>683</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F35" t="s">
         <v>765</v>
       </c>
-      <c r="G32">
+      <c r="G35">
         <v>12</v>
       </c>
-      <c r="L32" t="s">
+      <c r="L35" t="s">
         <v>766</v>
       </c>
-      <c r="Q32" t="s">
+      <c r="Q35" t="s">
         <v>687</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D33" t="s">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D36" t="s">
         <v>695</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F36" t="s">
         <v>767</v>
       </c>
-      <c r="G33">
+      <c r="G36">
         <v>8</v>
       </c>
-      <c r="L33" t="s">
+      <c r="L36" t="s">
         <v>756</v>
       </c>
-      <c r="P33" t="s">
+      <c r="P36" t="s">
         <v>697</v>
       </c>
-      <c r="Q33" t="s">
+      <c r="Q36" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D34" t="s">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D37" t="s">
         <v>695</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F37" t="s">
         <v>767</v>
       </c>
-      <c r="G34">
+      <c r="G37">
         <v>8</v>
       </c>
-      <c r="L34" t="s">
+      <c r="L37" t="s">
         <v>756</v>
       </c>
-      <c r="P34" t="s">
+      <c r="P37" t="s">
         <v>700</v>
       </c>
-      <c r="Q34" t="s">
+      <c r="Q37" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D35" t="s">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="D38" t="s">
         <v>703</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F38" t="s">
         <v>768</v>
       </c>
-      <c r="G35">
+      <c r="G38">
         <v>6</v>
       </c>
-      <c r="L35" t="s">
+      <c r="L38" t="s">
         <v>753</v>
       </c>
-      <c r="P35" t="s">
+      <c r="P38" t="s">
         <v>705</v>
       </c>
-      <c r="Q35" t="s">
+      <c r="Q38" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>708</v>
       </c>
-      <c r="G36">
+      <c r="G39">
         <v>6</v>
       </c>
-      <c r="P36" t="s">
+      <c r="P39" t="s">
         <v>710</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
         <v>713</v>
       </c>
-      <c r="G37">
+      <c r="G40">
         <v>36</v>
       </c>
-      <c r="P37" t="s">
+      <c r="P40" t="s">
         <v>715</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C38" t="s">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C41" t="s">
         <v>728</v>
       </c>
-      <c r="G38">
-        <v>1</v>
-      </c>
-      <c r="L38" t="s">
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="L41" t="s">
         <v>734</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C39" t="s">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C42" t="s">
         <v>729</v>
       </c>
-      <c r="G39">
-        <v>1</v>
-      </c>
-      <c r="L39" t="s">
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="L42" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C40" t="s">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C43" t="s">
         <v>730</v>
       </c>
-      <c r="G40">
-        <v>1</v>
-      </c>
-      <c r="L40" t="s">
+      <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="L43" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C41" t="s">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C44" t="s">
         <v>731</v>
       </c>
-      <c r="G41">
-        <v>1</v>
-      </c>
-      <c r="L41" t="s">
+      <c r="G44">
+        <v>1</v>
+      </c>
+      <c r="L44" t="s">
         <v>733</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F18" r:id="rId1" xr:uid="{1E990FAB-719E-432C-8625-A5212A735249}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
synch work local poistron to git
</commit_message>
<xml_diff>
--- a/data/NMD_Perturbation_TopStudySamples_20260712.xlsx
+++ b/data/NMD_Perturbation_TopStudySamples_20260712.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\aobermayer4\Projects\active\Public_NMD_Perturbation_Data\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://moffitt-my.sharepoint.com/personal/alyssa_obermayer_moffitt_org/Documents/Documents/Projects/Active/NMD_Perturbation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2586E139-F2AC-480F-9FE3-F3A5C02AEE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="13_ncr:1_{5A1180FC-E05E-412E-A9C8-872707654177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBB80609-CB8B-4057-A715-107CBCEA5C66}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DAD5C51E-F1D3-4296-A2F1-A74013D7D8F0}"/>
   </bookViews>
   <sheets>
     <sheet name="NMD_Perturbation_TopStudySample" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2395" uniqueCount="894">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2357" uniqueCount="866">
   <si>
     <t>GSE_ID</t>
   </si>
@@ -2620,97 +2620,13 @@
   </si>
   <si>
     <t>Also looked at NBAS siRNA as activator of UPF1</t>
-  </si>
-  <si>
-    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE176197</t>
-  </si>
-  <si>
-    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9108617/</t>
-  </si>
-  <si>
-    <t>PRJNA735254</t>
-  </si>
-  <si>
-    <t>Flp-In T-REx-293 cells</t>
-  </si>
-  <si>
-    <t>a specialized mammalian host line used for generating stable, isogenic cell lines with tightly regulated, inducible protein expression. They are ideal for high-level expression and functional studies of toxic or tightly controlled genes. [1, 2, 3, 4, 5]</t>
-  </si>
-  <si>
-    <t>GSE134059</t>
-  </si>
-  <si>
-    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE134059</t>
-  </si>
-  <si>
-    <t>PRJNA553576</t>
-  </si>
-  <si>
-    <t>SRP213944</t>
-  </si>
-  <si>
-    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE162699</t>
-  </si>
-  <si>
-    <t>PRJNA682628</t>
-  </si>
-  <si>
-    <t>SRP295982</t>
-  </si>
-  <si>
-    <t>GSE162699</t>
-  </si>
-  <si>
-    <t>GSE59884</t>
-  </si>
-  <si>
-    <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE59884</t>
-  </si>
-  <si>
-    <t>PRJNA256984</t>
-  </si>
-  <si>
-    <t>SRP045065</t>
-  </si>
-  <si>
-    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC4764554/</t>
-  </si>
-  <si>
-    <t>HEK-293T</t>
-  </si>
-  <si>
-    <t>non-targeting control siRNA or UPF1LL-specific siRNA were treated with vehicle control, puromycin, or thapsigargin</t>
-  </si>
-  <si>
-    <t>UPF1LL siRNA</t>
-  </si>
-  <si>
-    <t>HEK-293 Trex cells</t>
-  </si>
-  <si>
-    <t>overexpression of CLIP-tagged UPF1 isoforms 1 and 2 or GFP</t>
-  </si>
-  <si>
-    <t>UPF1LL/SL Overexpression</t>
-  </si>
-  <si>
-    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9108617/#embj2021108898-sec-0021</t>
-  </si>
-  <si>
-    <t>RIPseq, RNAseq</t>
-  </si>
-  <si>
-    <t>RNAseq</t>
-  </si>
-  <si>
-    <t>RIPseq</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2854,14 +2770,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3206,7 +3114,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="44">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -3250,9 +3158,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -3267,10 +3174,8 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="43"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="44">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -3304,7 +3209,6 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="43" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -3647,37 +3551,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E28C8A8-6FB1-4F0E-BBCF-A1462531D658}">
   <dimension ref="A1:AE80"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="32.5546875" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.44140625" customWidth="1"/>
-    <col min="10" max="12" width="20.88671875" customWidth="1"/>
-    <col min="13" max="13" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.88671875" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="32.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.42578125" customWidth="1"/>
+    <col min="10" max="12" width="20.85546875" customWidth="1"/>
+    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.85546875" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="20.88671875" customWidth="1"/>
-    <col min="28" max="28" width="23.88671875" customWidth="1"/>
-    <col min="29" max="29" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="20.88671875" customWidth="1"/>
+    <col min="17" max="17" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.85546875" customWidth="1"/>
+    <col min="28" max="28" width="23.85546875" customWidth="1"/>
+    <col min="29" max="29" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3769,7 +3673,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -3864,7 +3768,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -3959,7 +3863,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -4054,7 +3958,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
@@ -4149,7 +4053,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>28</v>
       </c>
@@ -4244,7 +4148,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -4339,7 +4243,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
@@ -4434,7 +4338,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>73</v>
       </c>
@@ -4529,7 +4433,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>73</v>
       </c>
@@ -4624,7 +4528,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>73</v>
       </c>
@@ -4719,7 +4623,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>73</v>
       </c>
@@ -4814,7 +4718,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>73</v>
       </c>
@@ -4909,7 +4813,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -5004,7 +4908,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>73</v>
       </c>
@@ -5099,7 +5003,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>73</v>
       </c>
@@ -5194,7 +5098,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5289,7 +5193,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>73</v>
       </c>
@@ -5384,7 +5288,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>73</v>
       </c>
@@ -5479,7 +5383,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>73</v>
       </c>
@@ -5574,7 +5478,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>73</v>
       </c>
@@ -5669,7 +5573,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>73</v>
       </c>
@@ -5764,7 +5668,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>73</v>
       </c>
@@ -5859,7 +5763,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>73</v>
       </c>
@@ -5954,7 +5858,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>73</v>
       </c>
@@ -6049,7 +5953,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>73</v>
       </c>
@@ -6144,7 +6048,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>150</v>
       </c>
@@ -6236,7 +6140,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>150</v>
       </c>
@@ -6328,7 +6232,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>150</v>
       </c>
@@ -6420,7 +6324,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>150</v>
       </c>
@@ -6512,7 +6416,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>150</v>
       </c>
@@ -6604,7 +6508,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>150</v>
       </c>
@@ -6696,7 +6600,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>150</v>
       </c>
@@ -6788,7 +6692,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>150</v>
       </c>
@@ -6880,7 +6784,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>150</v>
       </c>
@@ -6972,7 +6876,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>150</v>
       </c>
@@ -7064,7 +6968,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>150</v>
       </c>
@@ -7156,7 +7060,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>150</v>
       </c>
@@ -7248,7 +7152,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>150</v>
       </c>
@@ -7340,7 +7244,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>150</v>
       </c>
@@ -7432,7 +7336,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>206</v>
       </c>
@@ -7524,7 +7428,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>206</v>
       </c>
@@ -7616,7 +7520,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>206</v>
       </c>
@@ -7708,7 +7612,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>206</v>
       </c>
@@ -7800,7 +7704,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>206</v>
       </c>
@@ -7892,7 +7796,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>206</v>
       </c>
@@ -7984,7 +7888,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>206</v>
       </c>
@@ -8076,7 +7980,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>206</v>
       </c>
@@ -8168,7 +8072,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>206</v>
       </c>
@@ -8260,7 +8164,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>206</v>
       </c>
@@ -8352,7 +8256,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>206</v>
       </c>
@@ -8444,7 +8348,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>206</v>
       </c>
@@ -8536,7 +8440,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>206</v>
       </c>
@@ -8628,7 +8532,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>206</v>
       </c>
@@ -8720,7 +8624,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>206</v>
       </c>
@@ -8812,7 +8716,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>206</v>
       </c>
@@ -8904,7 +8808,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>206</v>
       </c>
@@ -8996,7 +8900,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>206</v>
       </c>
@@ -9088,7 +8992,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>206</v>
       </c>
@@ -9180,7 +9084,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>206</v>
       </c>
@@ -9272,7 +9176,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>311</v>
       </c>
@@ -9367,7 +9271,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>311</v>
       </c>
@@ -9462,7 +9366,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>311</v>
       </c>
@@ -9557,7 +9461,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>311</v>
       </c>
@@ -9652,7 +9556,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>311</v>
       </c>
@@ -9747,7 +9651,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>311</v>
       </c>
@@ -9842,7 +9746,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>311</v>
       </c>
@@ -9937,7 +9841,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>311</v>
       </c>
@@ -10032,7 +9936,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>311</v>
       </c>
@@ -10127,7 +10031,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>311</v>
       </c>
@@ -10222,7 +10126,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>311</v>
       </c>
@@ -10317,7 +10221,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>311</v>
       </c>
@@ -10412,7 +10316,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>348</v>
       </c>
@@ -10504,7 +10408,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>348</v>
       </c>
@@ -10593,7 +10497,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>348</v>
       </c>
@@ -10682,7 +10586,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>348</v>
       </c>
@@ -10771,7 +10675,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>348</v>
       </c>
@@ -10863,7 +10767,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>348</v>
       </c>
@@ -10952,7 +10856,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>348</v>
       </c>
@@ -11041,7 +10945,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:31" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>348</v>
       </c>
@@ -11138,21 +11042,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1739B9-C94C-4465-8F8F-0F3F742A5026}">
   <dimension ref="A1:R87"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.6640625" customWidth="1"/>
-    <col min="5" max="5" width="44.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="79.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="18" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" customWidth="1"/>
+    <col min="5" max="5" width="44.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="79.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="18" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11208,7 +11112,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -11258,7 +11162,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -11302,7 +11206,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>150</v>
       </c>
@@ -11352,7 +11256,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>457</v>
       </c>
@@ -11402,7 +11306,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>461</v>
       </c>
@@ -11452,7 +11356,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>206</v>
       </c>
@@ -11505,7 +11409,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>311</v>
       </c>
@@ -11558,7 +11462,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>348</v>
       </c>
@@ -11605,7 +11509,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>469</v>
       </c>
@@ -11655,7 +11559,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>474</v>
       </c>
@@ -11702,7 +11606,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>478</v>
       </c>
@@ -11755,7 +11659,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>483</v>
       </c>
@@ -11799,7 +11703,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>487</v>
       </c>
@@ -11843,7 +11747,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>492</v>
       </c>
@@ -11887,7 +11791,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>497</v>
       </c>
@@ -11934,7 +11838,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>501</v>
       </c>
@@ -11981,7 +11885,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>505</v>
       </c>
@@ -12025,7 +11929,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>508</v>
       </c>
@@ -12072,7 +11976,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>513</v>
       </c>
@@ -12116,7 +12020,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>516</v>
       </c>
@@ -12160,7 +12064,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>519</v>
       </c>
@@ -12204,7 +12108,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>522</v>
       </c>
@@ -12248,7 +12152,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>524</v>
       </c>
@@ -12295,7 +12199,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>526</v>
       </c>
@@ -12339,7 +12243,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>529</v>
       </c>
@@ -12389,7 +12293,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>532</v>
       </c>
@@ -12430,7 +12334,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>535</v>
       </c>
@@ -12477,7 +12381,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>539</v>
       </c>
@@ -12521,7 +12425,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>542</v>
       </c>
@@ -12565,7 +12469,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>545</v>
       </c>
@@ -12609,7 +12513,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>548</v>
       </c>
@@ -12653,7 +12557,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>551</v>
       </c>
@@ -12664,7 +12568,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>554</v>
       </c>
@@ -12675,7 +12579,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>557</v>
       </c>
@@ -12686,7 +12590,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>560</v>
       </c>
@@ -12697,7 +12601,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>563</v>
       </c>
@@ -12708,7 +12612,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>565</v>
       </c>
@@ -12719,7 +12623,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>567</v>
       </c>
@@ -12730,7 +12634,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>570</v>
       </c>
@@ -12741,7 +12645,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>573</v>
       </c>
@@ -12752,7 +12656,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>576</v>
       </c>
@@ -12763,7 +12667,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>579</v>
       </c>
@@ -12774,7 +12678,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>582</v>
       </c>
@@ -12785,7 +12689,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>585</v>
       </c>
@@ -12796,7 +12700,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>588</v>
       </c>
@@ -12807,7 +12711,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>591</v>
       </c>
@@ -12818,7 +12722,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>594</v>
       </c>
@@ -12829,7 +12733,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>596</v>
       </c>
@@ -12840,7 +12744,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>598</v>
       </c>
@@ -12851,7 +12755,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>600</v>
       </c>
@@ -12862,7 +12766,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>602</v>
       </c>
@@ -12873,7 +12777,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>604</v>
       </c>
@@ -12884,7 +12788,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>606</v>
       </c>
@@ -12895,7 +12799,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>608</v>
       </c>
@@ -12906,7 +12810,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>610</v>
       </c>
@@ -12917,7 +12821,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>612</v>
       </c>
@@ -12934,7 +12838,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>617</v>
       </c>
@@ -12951,7 +12855,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
         <v>621</v>
       </c>
@@ -12968,7 +12872,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
         <v>625</v>
       </c>
@@ -12985,7 +12889,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
         <v>629</v>
       </c>
@@ -13002,7 +12906,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>633</v>
       </c>
@@ -13019,7 +12923,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
         <v>637</v>
       </c>
@@ -13036,7 +12940,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>641</v>
       </c>
@@ -13053,7 +12957,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
         <v>645</v>
       </c>
@@ -13070,7 +12974,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
         <v>649</v>
       </c>
@@ -13087,7 +12991,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
         <v>653</v>
       </c>
@@ -13104,7 +13008,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
         <v>657</v>
       </c>
@@ -13121,7 +13025,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
         <v>661</v>
       </c>
@@ -13138,7 +13042,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
         <v>665</v>
       </c>
@@ -13155,7 +13059,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
         <v>669</v>
       </c>
@@ -13172,7 +13076,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>669</v>
       </c>
@@ -13189,7 +13093,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
         <v>675</v>
       </c>
@@ -13206,7 +13110,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
         <v>679</v>
       </c>
@@ -13223,7 +13127,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
         <v>683</v>
       </c>
@@ -13240,7 +13144,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
         <v>683</v>
       </c>
@@ -13257,7 +13161,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
         <v>33</v>
       </c>
@@ -13274,7 +13178,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
         <v>33</v>
       </c>
@@ -13291,7 +13195,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
         <v>33</v>
       </c>
@@ -13308,7 +13212,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
         <v>33</v>
       </c>
@@ -13325,7 +13229,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
         <v>695</v>
       </c>
@@ -13342,7 +13246,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
         <v>695</v>
       </c>
@@ -13359,7 +13263,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
         <v>703</v>
       </c>
@@ -13376,7 +13280,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
         <v>708</v>
       </c>
@@ -13393,7 +13297,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
         <v>713</v>
       </c>
@@ -13417,24 +13321,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89C31724-8146-4D7C-A3D2-DC7D492096E6}">
-  <dimension ref="A1:R44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:R41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.44140625" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" customWidth="1"/>
-    <col min="12" max="15" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" customWidth="1"/>
+    <col min="12" max="15" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>718</v>
       </c>
@@ -13490,7 +13394,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -13537,7 +13441,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -13581,7 +13485,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>150</v>
       </c>
@@ -13625,7 +13529,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>206</v>
       </c>
@@ -13669,7 +13573,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>311</v>
       </c>
@@ -13710,7 +13614,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>348</v>
       </c>
@@ -13754,7 +13658,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>469</v>
       </c>
@@ -13801,7 +13705,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>478</v>
       </c>
@@ -13842,7 +13746,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>483</v>
       </c>
@@ -13877,7 +13781,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>529</v>
       </c>
@@ -13915,7 +13819,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>612</v>
       </c>
@@ -13962,7 +13866,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>617</v>
       </c>
@@ -14006,7 +13910,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>621</v>
       </c>
@@ -14050,565 +13954,403 @@
         <v>865</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>625</v>
       </c>
-      <c r="B15" t="s">
-        <v>868</v>
-      </c>
-      <c r="C15" t="s">
-        <v>626</v>
-      </c>
-      <c r="E15" t="s">
-        <v>867</v>
-      </c>
-      <c r="F15" t="s">
-        <v>866</v>
-      </c>
       <c r="G15">
         <v>6</v>
       </c>
-      <c r="H15">
-        <v>3</v>
-      </c>
-      <c r="I15">
-        <v>3</v>
-      </c>
-      <c r="K15" t="s">
-        <v>424</v>
-      </c>
-      <c r="M15" t="s">
-        <v>778</v>
-      </c>
-      <c r="N15" t="s">
-        <v>869</v>
-      </c>
-      <c r="O15" t="s">
-        <v>870</v>
-      </c>
-      <c r="P15" t="s">
-        <v>893</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>871</v>
-      </c>
-      <c r="B16" t="s">
-        <v>873</v>
-      </c>
-      <c r="C16" t="s">
-        <v>874</v>
-      </c>
-      <c r="E16" t="s">
-        <v>890</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>872</v>
+        <v>629</v>
       </c>
       <c r="G16">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>633</v>
+      </c>
+      <c r="G17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>637</v>
+      </c>
+      <c r="G18">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>641</v>
+      </c>
+      <c r="F19" t="s">
+        <v>742</v>
+      </c>
+      <c r="G19">
+        <v>24</v>
+      </c>
+      <c r="L19" t="s">
+        <v>747</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>645</v>
+      </c>
+      <c r="F20" t="s">
+        <v>743</v>
+      </c>
+      <c r="G20">
+        <v>18</v>
+      </c>
+      <c r="L20" t="s">
+        <v>745</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D21" t="s">
+        <v>649</v>
+      </c>
+      <c r="F21" t="s">
+        <v>748</v>
+      </c>
+      <c r="G21">
         <v>15</v>
       </c>
-      <c r="H16">
-        <v>12</v>
-      </c>
-      <c r="I16">
-        <v>3</v>
-      </c>
-      <c r="K16" t="s">
-        <v>889</v>
-      </c>
-      <c r="L16" t="s">
-        <v>888</v>
-      </c>
-      <c r="M16" t="s">
-        <v>778</v>
-      </c>
-      <c r="N16" t="s">
-        <v>887</v>
-      </c>
-      <c r="P16" t="s">
-        <v>891</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>878</v>
-      </c>
-      <c r="B17" t="s">
-        <v>876</v>
-      </c>
-      <c r="C17" t="s">
-        <v>877</v>
-      </c>
-      <c r="E17" t="s">
-        <v>867</v>
-      </c>
-      <c r="F17" t="s">
-        <v>875</v>
-      </c>
-      <c r="G17">
-        <v>48</v>
-      </c>
-      <c r="H17">
-        <v>9</v>
-      </c>
-      <c r="I17">
-        <v>9</v>
-      </c>
-      <c r="J17">
-        <v>30</v>
-      </c>
-      <c r="K17" t="s">
-        <v>886</v>
-      </c>
-      <c r="L17" t="s">
-        <v>885</v>
-      </c>
-      <c r="M17" t="s">
-        <v>778</v>
-      </c>
-      <c r="N17" t="s">
-        <v>852</v>
-      </c>
-      <c r="P17" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>879</v>
-      </c>
-      <c r="B18" t="s">
-        <v>881</v>
-      </c>
-      <c r="C18" t="s">
-        <v>882</v>
-      </c>
-      <c r="E18" t="s">
-        <v>883</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>880</v>
-      </c>
-      <c r="G18">
-        <v>8</v>
-      </c>
-      <c r="H18">
-        <v>2</v>
-      </c>
-      <c r="I18">
-        <v>2</v>
-      </c>
-      <c r="J18">
-        <v>4</v>
-      </c>
-      <c r="K18" t="s">
-        <v>424</v>
-      </c>
-      <c r="M18" t="s">
-        <v>778</v>
-      </c>
-      <c r="N18" t="s">
-        <v>884</v>
-      </c>
-      <c r="P18" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>629</v>
-      </c>
-      <c r="G19">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>633</v>
-      </c>
-      <c r="G20">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>637</v>
-      </c>
-      <c r="G21">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="L21" t="s">
+        <v>750</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>641</v>
+        <v>653</v>
       </c>
       <c r="F22" t="s">
-        <v>742</v>
+        <v>751</v>
       </c>
       <c r="G22">
         <v>24</v>
       </c>
       <c r="L22" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="Q22" t="s">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
-        <v>645</v>
+        <v>657</v>
       </c>
       <c r="F23" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="G23">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="L23" t="s">
-        <v>745</v>
+        <v>756</v>
       </c>
       <c r="Q23" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
-        <v>649</v>
+        <v>661</v>
       </c>
       <c r="F24" t="s">
-        <v>748</v>
+        <v>757</v>
       </c>
       <c r="G24">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="L24" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="Q24" t="s">
-        <v>749</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>653</v>
+        <v>665</v>
       </c>
       <c r="F25" t="s">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="G25">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="L25" t="s">
         <v>753</v>
       </c>
       <c r="Q25" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>657</v>
+        <v>669</v>
       </c>
       <c r="F26" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="G26">
+        <v>18</v>
+      </c>
+      <c r="L26" t="s">
+        <v>762</v>
+      </c>
+      <c r="Q26" s="10" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
+        <v>669</v>
+      </c>
+      <c r="F27" t="s">
+        <v>761</v>
+      </c>
+      <c r="G27">
+        <v>18</v>
+      </c>
+      <c r="L27" t="s">
+        <v>762</v>
+      </c>
+      <c r="Q27" s="10" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>675</v>
+      </c>
+      <c r="F28" t="s">
+        <v>764</v>
+      </c>
+      <c r="G28">
+        <v>21</v>
+      </c>
+      <c r="L28" t="s">
+        <v>756</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D29" t="s">
+        <v>738</v>
+      </c>
+      <c r="F29" t="s">
+        <v>740</v>
+      </c>
+      <c r="G29">
         <v>27</v>
       </c>
-      <c r="L26" t="s">
+      <c r="L29" t="s">
+        <v>736</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D30" t="s">
+        <v>679</v>
+      </c>
+      <c r="F30" t="s">
+        <v>741</v>
+      </c>
+      <c r="G30">
+        <v>36</v>
+      </c>
+      <c r="L30" t="s">
+        <v>736</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D31" t="s">
+        <v>683</v>
+      </c>
+      <c r="F31" t="s">
+        <v>765</v>
+      </c>
+      <c r="G31">
+        <v>12</v>
+      </c>
+      <c r="L31" t="s">
+        <v>766</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>683</v>
+      </c>
+      <c r="F32" t="s">
+        <v>765</v>
+      </c>
+      <c r="G32">
+        <v>12</v>
+      </c>
+      <c r="L32" t="s">
+        <v>766</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>695</v>
+      </c>
+      <c r="F33" t="s">
+        <v>767</v>
+      </c>
+      <c r="G33">
+        <v>8</v>
+      </c>
+      <c r="L33" t="s">
         <v>756</v>
       </c>
-      <c r="Q26" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D27" t="s">
-        <v>661</v>
-      </c>
-      <c r="F27" t="s">
-        <v>757</v>
-      </c>
-      <c r="G27">
-        <v>24</v>
-      </c>
-      <c r="L27" t="s">
+      <c r="P33" t="s">
+        <v>697</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D34" t="s">
+        <v>695</v>
+      </c>
+      <c r="F34" t="s">
+        <v>767</v>
+      </c>
+      <c r="G34">
+        <v>8</v>
+      </c>
+      <c r="L34" t="s">
+        <v>756</v>
+      </c>
+      <c r="P34" t="s">
+        <v>700</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D35" t="s">
+        <v>703</v>
+      </c>
+      <c r="F35" t="s">
+        <v>768</v>
+      </c>
+      <c r="G35">
+        <v>6</v>
+      </c>
+      <c r="L35" t="s">
         <v>753</v>
       </c>
-      <c r="Q27" t="s">
+      <c r="P35" t="s">
+        <v>705</v>
+      </c>
+      <c r="Q35" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D28" t="s">
-        <v>665</v>
-      </c>
-      <c r="F28" t="s">
-        <v>759</v>
-      </c>
-      <c r="G28">
-        <v>9</v>
-      </c>
-      <c r="L28" t="s">
-        <v>753</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D29" t="s">
-        <v>669</v>
-      </c>
-      <c r="F29" t="s">
-        <v>761</v>
-      </c>
-      <c r="G29">
-        <v>18</v>
-      </c>
-      <c r="L29" t="s">
-        <v>762</v>
-      </c>
-      <c r="Q29" s="10" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D30" t="s">
-        <v>669</v>
-      </c>
-      <c r="F30" t="s">
-        <v>761</v>
-      </c>
-      <c r="G30">
-        <v>18</v>
-      </c>
-      <c r="L30" t="s">
-        <v>762</v>
-      </c>
-      <c r="Q30" s="10" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D31" t="s">
-        <v>675</v>
-      </c>
-      <c r="F31" t="s">
-        <v>764</v>
-      </c>
-      <c r="G31">
-        <v>21</v>
-      </c>
-      <c r="L31" t="s">
-        <v>756</v>
-      </c>
-      <c r="Q31" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D32" t="s">
-        <v>738</v>
-      </c>
-      <c r="F32" t="s">
-        <v>740</v>
-      </c>
-      <c r="G32">
-        <v>27</v>
-      </c>
-      <c r="L32" t="s">
-        <v>736</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>739</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D33" t="s">
-        <v>679</v>
-      </c>
-      <c r="F33" t="s">
-        <v>741</v>
-      </c>
-      <c r="G33">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>708</v>
+      </c>
+      <c r="G36">
+        <v>6</v>
+      </c>
+      <c r="P36" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>713</v>
+      </c>
+      <c r="G37">
         <v>36</v>
       </c>
-      <c r="L33" t="s">
-        <v>736</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D34" t="s">
-        <v>683</v>
-      </c>
-      <c r="F34" t="s">
-        <v>765</v>
-      </c>
-      <c r="G34">
-        <v>12</v>
-      </c>
-      <c r="L34" t="s">
-        <v>766</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>685</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D35" t="s">
-        <v>683</v>
-      </c>
-      <c r="F35" t="s">
-        <v>765</v>
-      </c>
-      <c r="G35">
-        <v>12</v>
-      </c>
-      <c r="L35" t="s">
-        <v>766</v>
-      </c>
-      <c r="Q35" t="s">
-        <v>687</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D36" t="s">
-        <v>695</v>
-      </c>
-      <c r="F36" t="s">
-        <v>767</v>
-      </c>
-      <c r="G36">
-        <v>8</v>
-      </c>
-      <c r="L36" t="s">
-        <v>756</v>
-      </c>
-      <c r="P36" t="s">
-        <v>697</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D37" t="s">
-        <v>695</v>
-      </c>
-      <c r="F37" t="s">
-        <v>767</v>
-      </c>
-      <c r="G37">
-        <v>8</v>
-      </c>
-      <c r="L37" t="s">
-        <v>756</v>
-      </c>
       <c r="P37" t="s">
-        <v>700</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="D38" t="s">
-        <v>703</v>
-      </c>
-      <c r="F38" t="s">
-        <v>768</v>
+        <v>715</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>728</v>
       </c>
       <c r="G38">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L38" t="s">
-        <v>753</v>
-      </c>
-      <c r="P38" t="s">
-        <v>705</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>708</v>
+        <v>734</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>729</v>
       </c>
       <c r="G39">
-        <v>6</v>
-      </c>
-      <c r="P39" t="s">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>713</v>
+        <v>1</v>
+      </c>
+      <c r="L39" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>730</v>
       </c>
       <c r="G40">
-        <v>36</v>
-      </c>
-      <c r="P40" t="s">
-        <v>715</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="L40" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C41" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="G41">
         <v>1</v>
       </c>
       <c r="L41" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C42" t="s">
-        <v>729</v>
-      </c>
-      <c r="G42">
-        <v>1</v>
-      </c>
-      <c r="L42" t="s">
-        <v>735</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C43" t="s">
-        <v>730</v>
-      </c>
-      <c r="G43">
-        <v>1</v>
-      </c>
-      <c r="L43" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C44" t="s">
-        <v>731</v>
-      </c>
-      <c r="G44">
-        <v>1</v>
-      </c>
-      <c r="L44" t="s">
         <v>733</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F18" r:id="rId1" xr:uid="{1E990FAB-719E-432C-8625-A5212A735249}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>